<commit_message>
refactor: pindahkan output excel ke folder p4 dan atur encoding console
</commit_message>
<xml_diff>
--- a/p4/hasil_cleaning.xlsx
+++ b/p4/hasil_cleaning.xlsx
@@ -446,270 +446,270 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Android 17 Resmi Meluncur, Ini HP Pertama yang Kebagian</t>
+          <t>Review iPhone 17e: Dipakai Ngonten dan Gaming, Susah Move On</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Android 17 Resmi Meluncur Ini HP Pertama yang Kebagian</t>
+          <t>Review iPhone 17e Dipakai Ngonten dan Gaming Susah Move On</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/consumer/d-8535083/android-17-resmi-meluncur-ini-hp-pertama-yang-kebagian</t>
+          <t>https://inet.detik.com/review-produk/d-8541015/review-iphone-17e-dipakai-ngonten-dan-gaming-susah-move-on</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>httpsinetdetikcomconsumerdandroidresmimeluncurinihppertamayangkebagian</t>
+          <t>httpsinetdetikcomreviewprodukdreviewiphoneedipakaingontendangamingsusahmoveon</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>17062026</t>
+          <t>21062026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Video: Xiaomi 17T Pro Udah Bisa Quickshare ke iPhone Tanpa Aplikasi Tambahan</t>
+          <t>China Perketat Ekspor Indium untuk Chip AI, Ini Fakta-faktanya</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Video Xiaomi 17T Pro Udah Bisa Quickshare ke iPhone Tanpa Aplikasi Tambahan</t>
+          <t>China Perketat Ekspor Indium untuk Chip AI Ini Faktafaktanya</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/detiktv/d-8535163/video-xiaomi-17t-pro-udah-bisa-quickshare-ke-iphone-tanpa-aplikasi-tambahan</t>
+          <t>https://inet.detik.com/cyberlife/d-8540924/china-perketat-ekspor-indium-untuk-chip-ai-ini-fakta-faktanya</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>httpsinetdetikcomdetiktvdvideoxiaomitproudahbisaquicksharekeiphonetanpaaplikasitambahan</t>
+          <t>httpsinetdetikcomcyberlifedchinaperketateksporindiumuntukchipaiinifaktafaktanya</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>17062026</t>
+          <t>21062026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Logitech G304 X Superlight &amp; G316 X 98 Hadir di RI, Gaming Makin Ngebut</t>
+          <t>Jadwal Kualifikasi Mobile Legends Asian Games Hari Ini: Indonesia Vs Kamboja</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Logitech G304 X Superlight G316 X 98 Hadir di RI Gaming Makin Ngebut</t>
+          <t>Jadwal Kualifikasi Mobile Legends Asian Games Hari Ini Indonesia Vs Kamboja</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/consumer/d-8534901/logitech-g304-x-superlight-g316-x-98-hadir-di-ri-gaming-makin-ngebut</t>
+          <t>https://inet.detik.com/esport/d-8540822/jadwal-kualifikasi-mobile-legends-asian-games-hari-ini-indonesia-vs-kamboja</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>httpsinetdetikcomconsumerdlogitechgxsuperlightgxhadirdirigamingmakinngebut</t>
+          <t>httpsinetdetikcomesportdjadwalkualifikasimobilelegendsasiangameshariiniindonesiavskamboja</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>17062026</t>
+          <t>21062026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>10 Foto Lionel Messi Hattrick, Dipuji Setinggi Langit</t>
+          <t>Norwegia Larang Anak SD Pakai AI Agar Tak Lupa Baca Tulis</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10 Foto Lionel Messi Hattrick Dipuji Setinggi Langit</t>
+          <t>Norwegia Larang Anak SD Pakai AI Agar Tak Lupa Baca Tulis</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/fotoinet/d-8535031/lionel-messi-hattrick-dipuji-setinggi-langit</t>
+          <t>https://inet.detik.com/cyberlife/d-8540819/norwegia-larang-anak-sd-pakai-ai-agar-tak-lupa-baca-tulis</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>httpsinetdetikcomfotoinetdlionelmessihattrickdipujisetinggilangit</t>
+          <t>httpsinetdetikcomcyberlifednorwegialaranganaksdpakaiaiagartaklupabacatulis</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>17062026</t>
+          <t>21062026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Kampus Ini Sudah Lahirkan 12 Unicorn AI dan Hardware, Ada DJI di Baliknya</t>
+          <t>Video: Truk Pantura-Spanduk Pecel Lele Inspirasi Google Doodle Ardhira Putra</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Kampus Ini Sudah Lahirkan 12 Unicorn AI dan Hardware Ada DJI di Baliknya</t>
+          <t>Video Truk PanturaSpanduk Pecel Lele Inspirasi Google Doodle Ardhira Putra</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8534903/kampus-ini-sudah-lahirkan-12-unicorn-ai-dan-hardware-ada-dji-di-baliknya</t>
+          <t>https://inet.detik.com/detiktv/d-8540793/video-truk-pantura-spanduk-pecel-lele-inspirasi-google-doodle-ardhira-putra</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>httpsinetdetikcomcyberlifedkampusinisudahlahirkanunicornaidanhardwareadadjidibaliknya</t>
+          <t>httpsinetdetikcomdetiktvdvideotrukpanturaspandukpecelleleinspirasigoogledoodleardhiraputra</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17062026</t>
+          <t>21062026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Zuckerberg Bayar Rp 248 T untuk Bocah Ajaib, Hasilnya Belum Ada</t>
+          <t>Gampang! Begini Cara Lacak Lokasi Orang Lewat WhatsApp dan Google Maps</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Zuckerberg Bayar Rp 248 T untuk Bocah Ajaib Hasilnya Belum Ada</t>
+          <t>Gampang Begini Cara Lacak Lokasi Orang Lewat WhatsApp dan Google Maps</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/business/d-8534912/zuckerberg-bayar-rp-248-t-untuk-bocah-ajaib-hasilnya-belum-ada</t>
+          <t>https://inet.detik.com/tips-dan-trik/d-8540747/gampang-begini-cara-lacak-lokasi-orang-lewat-whatsapp-dan-google-maps</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>httpsinetdetikcombusinessdzuckerbergbayarrptuntukbocahajaibhasilnyabelumada</t>
+          <t>httpsinetdetikcomtipsdantrikdgampangbeginicaralacaklokasioranglewatwhatsappdangooglemaps</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>17062026</t>
+          <t>21062026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>WhatsApp di iPhone Kini Bisa Pakai 2 Nomor Sekaligus, Begini Caranya</t>
+          <t>Microsoft Akan Cabut Dukungan Office 2021, Catat Tanggalnya!</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>WhatsApp di iPhone Kini Bisa Pakai 2 Nomor Sekaligus Begini Caranya</t>
+          <t>Microsoft Akan Cabut Dukungan Office 2021 Catat Tanggalnya</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/consumer/d-8534891/whatsapp-di-iphone-kini-bisa-pakai-2-nomor-sekaligus-begini-caranya</t>
+          <t>https://inet.detik.com/consumer/d-8540663/microsoft-akan-cabut-dukungan-office-2021-catat-tanggalnya</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>httpsinetdetikcomconsumerdwhatsappdiiphonekinibisapakainomorsekaligusbeginicaranya</t>
+          <t>httpsinetdetikcomconsumerdmicrosoftakancabutdukunganofficecatattanggalnya</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>17062026</t>
+          <t>21062026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Tak Sabar Tunggu GTA 6, Pria Ini Bikin Tiruannya Pakai AI</t>
+          <t>Proyek Raksasa di Gurun Nevada: 1.650 Antena untuk Mengintip Semesta</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tak Sabar Tunggu GTA 6 Pria Ini Bikin Tiruannya Pakai AI</t>
+          <t>Proyek Raksasa di Gurun Nevada 1650 Antena untuk Mengintip Semesta</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/games-news/d-8534872/tak-sabar-tunggu-gta-6-pria-ini-bikin-tiruannya-pakai-ai</t>
+          <t>https://inet.detik.com/science/d-8540606/proyek-raksasa-di-gurun-nevada-1-650-antena-untuk-mengintip-semesta</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>httpsinetdetikcomgamesnewsdtaksabartunggugtapriainibikintiruannyapakaiai</t>
+          <t>httpsinetdetikcomsciencedproyekraksasadigurunnevadaantenauntukmengintipsemesta</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>17062026</t>
+          <t>21062026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>15 Foto Hanya Mata Jeli yang Bisa Menemukan Sosok di Foto 'Penampakan' Ini</t>
+          <t>Samsung LED 50 UHD Smart TV Lebih Hemat Rp 1,8 Jutaan di Transmart Full Day Sale</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>15 Foto Hanya Mata Jeli yang Bisa Menemukan Sosok di Foto Penampakan Ini</t>
+          <t>Samsung LED 50 UHD Smart TV Lebih Hemat Rp 18 Jutaan di Transmart Full Day Sale</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/fotoinet/d-8534856/hanya-mata-jeli-yang-bisa-menemukan-sosok-di-foto-penampakan-ini</t>
+          <t>https://inet.detik.com/consumer/d-8540419/samsung-led-50-uhd-smart-tv-lebih-hemat-rp-1-8-jutaan-di-transmart-full-day-sale</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>httpsinetdetikcomfotoinetdhanyamatajeliyangbisamenemukansosokdifotopenampakanini</t>
+          <t>httpsinetdetikcomconsumerdsamsungleduhdsmarttvlebihhematrpjutaanditransmartfulldaysale</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>17062026</t>
+          <t>21062026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Haaland Menggila di Debut Piala Dunia 2026, Borong 2 Gol Bikin Heboh Medsos</t>
+          <t>Transmart Full Day Sale Diskon Gede, Kulkas Polytron 436L Hemat Jutaan</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Haaland Menggila di Debut Piala Dunia 2026 Borong 2 Gol Bikin Heboh Medsos</t>
+          <t>Transmart Full Day Sale Diskon Gede Kulkas Polytron 436L Hemat Jutaan</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8534834/haaland-menggila-di-debut-piala-dunia-2026-borong-2-gol-bikin-heboh-medsos</t>
+          <t>https://inet.detik.com/consumer/d-8540418/transmart-full-day-sale-diskon-gede-kulkas-polytron-436l-hemat-jutaan</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>httpsinetdetikcomcyberlifedhaalandmenggiladidebutpialaduniaboronggolbikinhebohmedsos</t>
+          <t>httpsinetdetikcomconsumerdtransmartfulldaysalediskongedekulkaspolytronlhematjutaan</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>17062026</t>
+          <t>21062026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
menambahkan scraping isi berita, cleaning data, export excel, dan perbaikan tampilan web berita
</commit_message>
<xml_diff>
--- a/p4/hasil_cleaning.xlsx
+++ b/p4/hasil_cleaning.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Hasil Cleaning" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,10 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -49,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,339 +413,257 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>judul_asli</t>
+          <t>Judul_Raw</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>judul_clean</t>
+          <t>Waktu_Public_Raw</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>url_link</t>
+          <t>Judul_Clean</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>url_link_clean</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url_gambar</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>waktu_scraping</t>
+          <t>Waktu_Public_Clean</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AI Masuk Program Bansos, Komdigi Bidik 50 Juta Penerima Manfaat</t>
+          <t xml:space="preserve">  AI Ada di Mana-mana, Traffic Internet Diramal Naik 5 Kali Lipat  </t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AI Masuk Program Bansos, Komdigi Bidik 50 Juta Penerima Manfaat</t>
+          <t>18 Mei 2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8543282/ai-masuk-program-bansos-komdigi-bidik-50-juta-penerima-manfaat</t>
+          <t>AI Ada Di Mana-mana, Traffic Internet Diramal Naik 5 Kali Lipat</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8543282/ai-masuk-program-bansos-komdigi-bidik-50-juta-penerima-manfaat</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/23/menkomdigi-1782187642616_43.jpeg?w=250&amp;q=90</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="n">
-        <v>46196.58473109645</v>
+          <t>20260518</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>10 Foto Meme Lionel Messi Dikasih Mahkota oleh Miroslav Klose</t>
+          <t>Menkomdigi:   Transformasi Digital RI Harus Dibangun Secara Komunal</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>10 Foto Meme Lionel Messi Dikasih Mahkota oleh Miroslav Klose</t>
+          <t>19 Mei 2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/fotoinet/d-8543160/meme-lionel-messi-dikasih-mahkota-oleh-miroslav-klose</t>
+          <t>Menkomdigi: Transformasi Digital RI Harus Dibangun Secara Komunal</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/fotoinet/d-8543160/meme-lionel-messi-dikasih-mahkota-oleh-miroslav-klose</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/23/meme-messi-1782182261909_43.png?w=250&amp;q=90</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="n">
-        <v>46196.58473109645</v>
+          <t>20260519</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Eropa Mendidih Akibat Gelombang Panas, Suhu Tembus 42 Derajat</t>
+          <t xml:space="preserve">	19% Penduduk RI Belum Terhubung Internet, Ini Janji Pemerintah</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Eropa Mendidih Akibat Gelombang Panas, Suhu Tembus 42 Derajat</t>
+          <t>20 Mei 2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/science/d-8543117/eropa-mendidih-akibat-gelombang-panas-suhu-tembus-42-derajat</t>
+          <t>19% Penduduk RI Belum Terhubung Internet, Ini Janji Pemerintah</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/science/d-8543117/eropa-mendidih-akibat-gelombang-panas-suhu-tembus-42-derajat</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/22/gelombang-panas-eropa-transportasi-dan-acara-dibatalkan-1782111178564_43.jpeg?w=250&amp;q=90</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="n">
-        <v>46196.58473109645</v>
+          <t>20260520</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Heboh! Aplikasi Peta Ini Ungkap Data Rahasia Wilayah Korea Utara</t>
+          <t>Beli Nomor HP Baru Tak Cukup NIK, Pekan Depan Wajib Verifikasi Wajah</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Heboh! Aplikasi Peta Ini Ungkap Data Rahasia Wilayah Korea Utara</t>
+          <t>21 Mei 2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8543091/heboh-aplikasi-peta-ini-ungkap-data-rahasia-wilayah-korea-utara</t>
+          <t>Beli Nomor HP Baru Tak Cukup NIK, Pekan Depan Wajib Verifikasi Wajah</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8543091/heboh-aplikasi-peta-ini-ungkap-data-rahasia-wilayah-korea-utara</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2025/09/03/kereta-yang-dinaiki-kim-jong-un-dari-korea-utara-menuju-beijing-chnia-untuk-menghadiri-parade-militer-1756891002533_43.jpeg?w=250&amp;q=90</t>
-        </is>
-      </c>
-      <c r="F5" s="1" t="n">
-        <v>46196.58473109645</v>
+          <t>20260521</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Messi Jadi Top Skor Piala Dunia Sepanjang Masa, Google Ikut Berpesta</t>
+          <t xml:space="preserve"> Satelit Jadi Kunci Pemerataan Akses Digital hingga Pelosok RI </t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Messi Jadi Top Skor Piala Dunia Sepanjang Masa, Google Ikut Berpesta</t>
+          <t>22 Mei 2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8543090/messi-jadi-top-skor-piala-dunia-sepanjang-masa-google-ikut-berpesta</t>
+          <t>Satelit Jadi Kunci Pemerataan Akses Digital Hingga Pelosok RI</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8543090/messi-jadi-top-skor-piala-dunia-sepanjang-masa-google-ikut-berpesta</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/21/undav-meledak-dan-samai-messi-perebutan-top-skor-pildun-2026-makin-panas-1782004747819_43.jpeg?w=250&amp;q=90</t>
-        </is>
-      </c>
-      <c r="F6" s="1" t="n">
-        <v>46196.58473109645</v>
+          <t>20260522</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Tecno Camon Slim Meluncur, HP 6,39 mm dengan LED Kreatif Unik</t>
+          <t>Schneider OffGrid Rilis di RI, Power Station untuk Kemah &amp; Listrik Padam</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Tecno Camon Slim Meluncur, HP 6,39 mm dengan LED Kreatif Unik</t>
+          <t>23 Mei 2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/consumer/d-8543081/tecno-camon-slim-meluncur-hp-6-39-mm-dengan-led-kreatif-unik</t>
+          <t>Schneider Offgrid Rilis Di RI, Power Station Untuk Kemah &amp; Listrik Padam</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/consumer/d-8543081/tecno-camon-slim-meluncur-hp-6-39-mm-dengan-led-kreatif-unik</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/23/tecno-camon-slim-1782177580666_43.png?w=250&amp;q=90</t>
-        </is>
-      </c>
-      <c r="F7" s="1" t="n">
-        <v>46196.58473109645</v>
+          <t>20260523</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>10 Foto Tim IT Menangis! Foto-foto Instalasi Kabel Ini Bikin Geleng Kepala</t>
+          <t>AMD dan Intel Garap ACE Buat Tantang Dominasi Nvidia di AI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>10 Foto Tim IT Menangis! Foto-foto Instalasi Kabel Ini Bikin Geleng Kepala</t>
+          <t>24 Mei 2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/fotoinet/d-8543055/tim-it-menangis-foto-foto-instalasi-kabel-ini-bikin-geleng-kepala</t>
+          <t>AMD Dan Intel Garap ACE Buat Tantang Dominasi Nvidia Di AI</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/fotoinet/d-8543055/tim-it-menangis-foto-foto-instalasi-kabel-ini-bikin-geleng-kepala</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/23/instalasi-kabel-bikin-tim-it-menangis-1782176504867_43.jpeg?w=250&amp;q=90</t>
-        </is>
-      </c>
-      <c r="F8" s="1" t="n">
-        <v>46196.58473109645</v>
+          <t>20260524</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Mbappe Lewati Messi, 15 Gol Piala Dunia Tercepat Tuai Pujian Selangit</t>
+          <t>Smartphone Bagus    Bukan Cuma Soal Harga</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Mbappe Lewati Messi, 15 Gol Piala Dunia Tercepat Tuai Pujian Selangit</t>
+          <t>25 Mei 2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8543043/mbappe-lewati-messi-15-gol-piala-dunia-tercepat-tuai-pujian-selangit</t>
+          <t>Smartphone Bagus Bukan Cuma Soal Harga</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8543043/mbappe-lewati-messi-15-gol-piala-dunia-tercepat-tuai-pujian-selangit</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/17/kylian-mbappe-1781648830427_43.jpeg?w=250&amp;q=90</t>
-        </is>
-      </c>
-      <c r="F9" s="1" t="n">
-        <v>46196.58473109645</v>
+          <t>20260525</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ingat! Aturan Daftar Nomor HP Baru Berlaku Pekan Depan</t>
+          <t xml:space="preserve">
+Telkomsel Ubah Ribuan Langkah di Digiland Run 2026 Jadi Pohon Mangrove
+</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Ingat! Aturan Daftar Nomor HP Baru Berlaku Pekan Depan</t>
+          <t>26 Mei 2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/law-and-policy/d-8543024/ingat-aturan-daftar-nomor-hp-baru-berlaku-pekan-depan</t>
+          <t>Telkomsel Ubah Ribuan Langkah Di Digiland Run 2026 Jadi Pohon Mangrove</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/law-and-policy/d-8543024/ingat-aturan-daftar-nomor-hp-baru-berlaku-pekan-depan</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2025/11/26/ilustrasi-face-recognition-1764163471563_43.jpeg?w=250&amp;q=90</t>
-        </is>
-      </c>
-      <c r="F10" s="1" t="n">
-        <v>46196.58473109645</v>
+          <t>20260526</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Messi Ukir 4 Rekor Baru Piala Dunia Sekaligus, Status GOAT Kian Kokoh</t>
+          <t>Shin Ye Eun Meriahkan Housewarming by LG di Indonesia</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Messi Ukir 4 Rekor Baru Piala Dunia Sekaligus, Status GOAT Kian Kokoh</t>
+          <t>27 Mei 2026</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8543019/messi-ukir-4-rekor-baru-piala-dunia-sekaligus-status-goat-kian-kokoh</t>
+          <t>Shin Ye Eun Meriahkan Housewarming By LG Di Indonesia</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8543019/messi-ukir-4-rekor-baru-piala-dunia-sekaligus-status-goat-kian-kokoh</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/23/lionel-messi-timnas-argentina-piala-dunia-2026-argentina-vs-austria-top-skor-piala-dunia-1782157290513_43.jpeg?w=250&amp;q=90</t>
-        </is>
-      </c>
-      <c r="F11" s="1" t="n">
-        <v>46196.58473109645</v>
+          <t>20260527</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>